<commit_message>
Standard program written for each house; sample menu and bar check; handbook and steps of service optional; targets from POS history
</commit_message>
<xml_diff>
--- a/packages/web/public/templates/blm-client-intake.xlsx
+++ b/packages/web/public/templates/blm-client-intake.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +70,10 @@
       <color rgb="006E675E"/>
       <sz val="10"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="008B8277"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -101,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -129,6 +133,9 @@
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -218,7 +225,7 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Net sales divided by tickets, in dollars.</t>
+        <t>Net sales divided by tickets. Blank and BLM sets it from your POS exports.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -648,7 +655,7 @@
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2.  Stores: one row per restaurant. Your spend per ticket targets for dinner and lunch, and the links to your review pages.</t>
+          <t>2.  Stores: one row per restaurant, with the links to your review pages. Targets are optional: leave them blank and BLM sets them from your POS sales exports with you.</t>
         </is>
       </c>
     </row>
@@ -669,7 +676,7 @@
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>5.  Material: tell us which menus, lists and manuals you have, and how you will send them.</t>
+          <t>5.  Material: tell us which menus, lists and manuals you have, and how you will send them. A handbook is optional; no handbook is fine.</t>
         </is>
       </c>
     </row>
@@ -966,16 +973,16 @@
         </is>
       </c>
       <c r="D2" s="11" t="n">
-        <v>175</v>
+        <v>78</v>
       </c>
       <c r="E2" s="11" t="n">
-        <v>160</v>
+        <v>73</v>
       </c>
       <c r="F2" s="11" t="n">
-        <v>95</v>
+        <v>64</v>
       </c>
       <c r="G2" s="11" t="n">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="H2" s="11" t="n">
         <v>16</v>
@@ -16764,13 +16771,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -16794,6 +16802,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Why we ask</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
@@ -16801,6 +16814,11 @@
           <t>Food menu</t>
         </is>
       </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>Needed. Every dish, its story and its allergens become the menu module and its check.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -16808,6 +16826,11 @@
           <t>Wine list</t>
         </is>
       </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>Needed. By the glass and bottles become the wine module, pairings and the wine check.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -16815,6 +16838,11 @@
           <t>Bar and cocktail menu</t>
         </is>
       </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Needed. Your cocktails, spirits and beers become the bar modules and their checks.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -16822,6 +16850,11 @@
           <t>Steps of service</t>
         </is>
       </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>Optional. If you have none, or yours is out of date, we use the BLM standard steps.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -16829,6 +16862,11 @@
           <t>House standards or handbook</t>
         </is>
       </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>Optional. Many houses have none, or an old one. Tell us your rules in Notes and we write them in.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -16836,11 +16874,21 @@
           <t>Allergy, safety and comp protocols</t>
         </is>
       </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>Optional. The BLM standard is used until yours arrive.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>POS screenshots or walkthrough</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>Optional. Only if you want a check on your own POS screens.</t>
         </is>
       </c>
     </row>

</xml_diff>